<commit_message>
Update inventory for Jeddah - 1784521461989
</commit_message>
<xml_diff>
--- a/stores/Jeddah.xlsx
+++ b/stores/Jeddah.xlsx
@@ -126,6 +126,38 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t>6941205320866</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr" s="2">
+        <is>
+          <t>1-2-3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update inventory for Jeddah - 1784523376377
</commit_message>
<xml_diff>
--- a/stores/Jeddah.xlsx
+++ b/stores/Jeddah.xlsx
@@ -158,6 +158,38 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t>038949984204</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t>1-2-3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>